<commit_message>
PDF cliente nuevo con condiciones de pago, muebles desactivables y recargo sobre el total
- PDF cliente con color: cabecera, tabla por mueble, base imponible, IVA,
  total y condiciones de aceptación (pago inicial y número de cuenta)
- Casilla Incluir en cada mueble para dejarlo fuera del presupuesto
- El recargo por escala se calcula sobre el total con acabado y se puede desactivar
- Parámetros nuevos en el catálogo: pago inicial (%) y número de cuenta

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MHBE3gE6AFc5rMzkXkJrid
</commit_message>
<xml_diff>
--- a/catalogo.xlsx
+++ b/catalogo.xlsx
@@ -6061,7 +6061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6179,7 +6179,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12">
@@ -6209,6 +6209,28 @@
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Pago inicial al aceptar (%)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Número de cuenta (IBAN)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ESXX XXXX XXXX XXXX XXXX XXXX</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>